<commit_message>
actualizacion del script de aventes para agosto
</commit_message>
<xml_diff>
--- a/REPORTE_ADUANAL_SANOFI_2026_01_2026_12.xlsx
+++ b/REPORTE_ADUANAL_SANOFI_2026_01_2026_12.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q90"/>
+  <dimension ref="A1:Q93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1636,27 +1636,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Exportación</t>
+          <t>Importación</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>240</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MNSE261396</t>
+          <t>LT2697801</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>6002651</t>
+          <t>6003315</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1666,66 +1666,66 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>26/08/2026</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>D142139</t>
+          <t>A60610</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>A9421A2A-7B8C-497F-9BA4-2F89B766F19F</t>
+          <t>DC690F97-E5F2-466D-B378-230DA32E2527</t>
         </is>
       </c>
       <c r="N18" t="n">
-        <v>1425.93</v>
+        <v>1360</v>
       </c>
       <c r="O18" t="n">
-        <v>228.15</v>
+        <v>217.6</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>1425.93</v>
+        <v>1577.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Exportación</t>
+          <t>Importación</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>240</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MNSE261396</t>
+          <t>LT2697801</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>6002651</t>
+          <t>6003315</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1735,31 +1735,26 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>21/08/2026</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>D142139</t>
+          <t>130175</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AGENCIA ADUANAL ALVELAIS ALARCON S.C.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>E4F1F3DF-2F1B-4F79-B5AB-47332D1EC146</t>
+          <t>GASTOS LADO AMERICANO</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>1989.17</v>
+        <v>7312.2</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -1768,33 +1763,33 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>1989.17</v>
+        <v>7312.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exportación</t>
+          <t>Importación</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>240</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MNSE261396</t>
+          <t>LT2697801</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>6002651</t>
+          <t>6003315</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1804,12 +1799,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>A44374</t>
+          <t>A50513</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1824,26 +1819,26 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>7eec3776-ccc7-4268-884d-0cc33a3e6aa9</t>
+          <t>254b12fe-c46a-47ac-8441-8705cff2f830</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>10505.1</v>
+        <v>6160</v>
       </c>
       <c r="O20" t="n">
-        <v>1680.82</v>
+        <v>985.6</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>12185.92</v>
+        <v>7145.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Importación</t>
+          <t>Exportación</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1858,12 +1853,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MNSI259435</t>
+          <t>MNSE261396</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>5012652</t>
+          <t>6002651</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1873,46 +1868,46 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>13/01/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>A55103</t>
+          <t>D142139</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>A3E52A2D-3327-4DE7-8BA1-D4DEC98336CF</t>
+          <t>A9421A2A-7B8C-497F-9BA4-2F89B766F19F</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>3250</v>
+        <v>1425.93</v>
       </c>
       <c r="O21" t="n">
-        <v>520</v>
+        <v>228.15</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>3770</v>
+        <v>1425.93</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Importación</t>
+          <t>Exportación</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1927,12 +1922,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MNSI259435</t>
+          <t>MNSE261396</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5012652</t>
+          <t>6002651</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1942,12 +1937,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>D140092</t>
+          <t>D142139</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1962,26 +1957,26 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>434a24fc-e626-44dd-af33-3592cb71d32c</t>
+          <t>E4F1F3DF-2F1B-4F79-B5AB-47332D1EC146</t>
         </is>
       </c>
       <c r="N22" t="n">
-        <v>39417.44</v>
+        <v>1989.17</v>
       </c>
       <c r="O22" t="n">
-        <v>6306.79</v>
+        <v>0</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>39417.44</v>
+        <v>1989.17</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Importación</t>
+          <t>Exportación</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1996,12 +1991,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MNSI259435</t>
+          <t>MNSE261396</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>5012652</t>
+          <t>6002651</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2011,40 +2006,40 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>06/01/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>D140092</t>
+          <t>A44374</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>E40F62F4-F348-50B4-91FC-0991187A6A12</t>
+          <t>7eec3776-ccc7-4268-884d-0cc33a3e6aa9</t>
         </is>
       </c>
       <c r="N23" t="n">
-        <v>5300</v>
+        <v>10505.1</v>
       </c>
       <c r="O23" t="n">
-        <v>848</v>
+        <v>1680.82</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>5300</v>
+        <v>12185.92</v>
       </c>
     </row>
     <row r="24">
@@ -2080,40 +2075,40 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>13/01/2026</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>A41636</t>
+          <t>A55103</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>HONORARIOS DE AGENCIA</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>5e1da7e1-52c6-42fc-a495-0d36a1e318ad</t>
+          <t>A3E52A2D-3327-4DE7-8BA1-D4DEC98336CF</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>52967.44</v>
+        <v>3250</v>
       </c>
       <c r="O24" t="n">
-        <v>8474.790000000001</v>
+        <v>520</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>61442.23</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="25">
@@ -2134,12 +2129,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MNSI259829</t>
+          <t>MNSI259435</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>5012757</t>
+          <t>5012652</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2149,40 +2144,40 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>13/01/2026</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>A55104</t>
+          <t>D140092</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>752A45FB-B26F-4101-925F-8540282E2FA8</t>
+          <t>434a24fc-e626-44dd-af33-3592cb71d32c</t>
         </is>
       </c>
       <c r="N25" t="n">
-        <v>3250</v>
+        <v>39417.44</v>
       </c>
       <c r="O25" t="n">
-        <v>520</v>
+        <v>6306.79</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>3770</v>
+        <v>39417.44</v>
       </c>
     </row>
     <row r="26">
@@ -2203,12 +2198,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MNSI259829</t>
+          <t>MNSI259435</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>5012757</t>
+          <t>5012652</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2223,35 +2218,35 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>A733</t>
+          <t>D140092</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>ETX SERVICIOS LOGISTICOS INTEGRALES</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>aefcfe8d-46f5-406e-a0c6-ee7d3be63d2f</t>
+          <t>E40F62F4-F348-50B4-91FC-0991187A6A12</t>
         </is>
       </c>
       <c r="N26" t="n">
-        <v>55000</v>
+        <v>5300</v>
       </c>
       <c r="O26" t="n">
-        <v>8800</v>
+        <v>848</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>63800</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="27">
@@ -2272,12 +2267,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MNSI259829</t>
+          <t>MNSI259435</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>5012757</t>
+          <t>5012652</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2287,40 +2282,40 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>27/12/2025</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>D139911</t>
+          <t>A41636</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>10E5EDDA-552C-4832-961D-FDB2E02F8078</t>
+          <t>5e1da7e1-52c6-42fc-a495-0d36a1e318ad</t>
         </is>
       </c>
       <c r="N27" t="n">
-        <v>1767</v>
+        <v>52967.44</v>
       </c>
       <c r="O27" t="n">
-        <v>282.72</v>
+        <v>8474.790000000001</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>1767</v>
+        <v>61442.23</v>
       </c>
     </row>
     <row r="28">
@@ -2356,40 +2351,40 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>13/01/2026</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>D139911</t>
+          <t>A55104</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>76D407D9-6E3E-4D1F-AD75-64C612D27054</t>
+          <t>752A45FB-B26F-4101-925F-8540282E2FA8</t>
         </is>
       </c>
       <c r="N28" t="n">
-        <v>1392</v>
+        <v>3250</v>
       </c>
       <c r="O28" t="n">
-        <v>222.72</v>
+        <v>520</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>1392</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="29">
@@ -2425,40 +2420,40 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>D139911</t>
+          <t>A733</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>ETX SERVICIOS LOGISTICOS INTEGRALES</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>88820473-E723-4B04-BE68-90920154E56A</t>
+          <t>aefcfe8d-46f5-406e-a0c6-ee7d3be63d2f</t>
         </is>
       </c>
       <c r="N29" t="n">
-        <v>487</v>
+        <v>55000</v>
       </c>
       <c r="O29" t="n">
-        <v>77.92</v>
+        <v>8800</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>487</v>
+        <v>63800</v>
       </c>
     </row>
     <row r="30">
@@ -2494,7 +2489,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>27/12/2025</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2514,20 +2509,20 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>55AF2698-D6BE-4A88-8E4A-9AE967A15C95</t>
+          <t>10E5EDDA-552C-4832-961D-FDB2E02F8078</t>
         </is>
       </c>
       <c r="N30" t="n">
-        <v>11135</v>
+        <v>1767</v>
       </c>
       <c r="O30" t="n">
-        <v>1781.6</v>
+        <v>282.72</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>11135</v>
+        <v>1767</v>
       </c>
     </row>
     <row r="31">
@@ -2563,7 +2558,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>31/12/2025</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2583,20 +2578,20 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>B8E26BEA-1819-4A79-BB25-65499A4D9EC4</t>
+          <t>76D407D9-6E3E-4D1F-AD75-64C612D27054</t>
         </is>
       </c>
       <c r="N31" t="n">
-        <v>2226</v>
+        <v>1392</v>
       </c>
       <c r="O31" t="n">
-        <v>356.16</v>
+        <v>222.72</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>2226</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="32">
@@ -2632,7 +2627,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>05/01/2026</t>
+          <t>31/12/2025</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2652,20 +2647,20 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>7D3C31D8-A1C3-4CC4-AC68-4AE7248C6D95</t>
+          <t>88820473-E723-4B04-BE68-90920154E56A</t>
         </is>
       </c>
       <c r="N32" t="n">
-        <v>47026.76</v>
+        <v>487</v>
       </c>
       <c r="O32" t="n">
-        <v>7524.28</v>
+        <v>77.92</v>
       </c>
       <c r="P32" t="n">
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>47026.76</v>
+        <v>487</v>
       </c>
     </row>
     <row r="33">
@@ -2701,7 +2696,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>26/12/2025</t>
+          <t>31/12/2025</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2716,25 +2711,25 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>D252FB29-584D-4EB5-B92C-BFC4331F0697</t>
+          <t>55AF2698-D6BE-4A88-8E4A-9AE967A15C95</t>
         </is>
       </c>
       <c r="N33" t="n">
-        <v>1000</v>
+        <v>11135</v>
       </c>
       <c r="O33" t="n">
-        <v>160</v>
+        <v>1781.6</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>1000</v>
+        <v>11135</v>
       </c>
     </row>
     <row r="34">
@@ -2770,7 +2765,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>23/12/2025</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2785,25 +2780,25 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>1D2D8EB7-5E14-445B-B1AA-3788F12B2C39</t>
+          <t>B8E26BEA-1819-4A79-BB25-65499A4D9EC4</t>
         </is>
       </c>
       <c r="N34" t="n">
-        <v>20250</v>
+        <v>2226</v>
       </c>
       <c r="O34" t="n">
-        <v>3240</v>
+        <v>356.16</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>20250</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="35">
@@ -2839,40 +2834,40 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>15/01/2026</t>
+          <t>05/01/2026</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>A41583</t>
+          <t>D139911</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>HONORARIOS DE AGENCIA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>c9d79cd7-5b16-46d8-bda9-abd6250d72f3</t>
+          <t>7D3C31D8-A1C3-4CC4-AC68-4AE7248C6D95</t>
         </is>
       </c>
       <c r="N35" t="n">
-        <v>148533.76</v>
+        <v>47026.76</v>
       </c>
       <c r="O35" t="n">
-        <v>23765.4</v>
+        <v>7524.28</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>172299.16</v>
+        <v>47026.76</v>
       </c>
     </row>
     <row r="36">
@@ -2883,7 +2878,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2893,12 +2888,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>MNSI261767</t>
+          <t>MNSI259829</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>6002723</t>
+          <t>5012757</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2908,40 +2903,40 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>26/12/2025</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>A57321</t>
+          <t>D139911</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>90D48494-66CE-4107-86BC-B2DA79CD6177</t>
+          <t>D252FB29-584D-4EB5-B92C-BFC4331F0697</t>
         </is>
       </c>
       <c r="N36" t="n">
-        <v>6500</v>
+        <v>1000</v>
       </c>
       <c r="O36" t="n">
-        <v>1040</v>
+        <v>160</v>
       </c>
       <c r="P36" t="n">
         <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>7540</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="37">
@@ -2952,7 +2947,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2962,12 +2957,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>MNSI261767</t>
+          <t>MNSI259829</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>6002723</t>
+          <t>5012757</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2977,40 +2972,40 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>FM013590</t>
+          <t>D139911</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>131D5A70-FCAA-6D46-9B4F-5655A1097276</t>
+          <t>1D2D8EB7-5E14-445B-B1AA-3788F12B2C39</t>
         </is>
       </c>
       <c r="N37" t="n">
-        <v>44000</v>
+        <v>20250</v>
       </c>
       <c r="O37" t="n">
-        <v>7040</v>
+        <v>3240</v>
       </c>
       <c r="P37" t="n">
-        <v>1760</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>49280</v>
+        <v>20250</v>
       </c>
     </row>
     <row r="38">
@@ -3021,7 +3016,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+          <t>SANOFI - AVENTIS DE MEXICO, S.A. DE C.V.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3031,12 +3026,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MNSI261767</t>
+          <t>MNSI259829</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6002723</t>
+          <t>5012757</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3046,40 +3041,40 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>15/01/2026</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>FM013591</t>
+          <t>A41583</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>BA8E4D43-500F-614F-815A-935A4AA73678</t>
+          <t>c9d79cd7-5b16-46d8-bda9-abd6250d72f3</t>
         </is>
       </c>
       <c r="N38" t="n">
-        <v>44000</v>
+        <v>148533.76</v>
       </c>
       <c r="O38" t="n">
-        <v>7040</v>
+        <v>23765.4</v>
       </c>
       <c r="P38" t="n">
-        <v>1760</v>
+        <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>49280</v>
+        <v>172299.16</v>
       </c>
     </row>
     <row r="39">
@@ -3115,40 +3110,40 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>FM013648</t>
+          <t>A57321</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>ESTADIAS</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>8CCE2D32-B553-354A-BC06-82B7A4BB3BCF</t>
+          <t>90D48494-66CE-4107-86BC-B2DA79CD6177</t>
         </is>
       </c>
       <c r="N39" t="n">
-        <v>38500</v>
+        <v>6500</v>
       </c>
       <c r="O39" t="n">
-        <v>6160</v>
+        <v>1040</v>
       </c>
       <c r="P39" t="n">
         <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>44660</v>
+        <v>7540</v>
       </c>
     </row>
     <row r="40">
@@ -3189,7 +3184,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>FM013649</t>
+          <t>FM013590</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3199,25 +3194,25 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>ESTADIAS</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>103BB1B9-B764-D245-BAA7-3A9B0C7B44DC</t>
+          <t>131D5A70-FCAA-6D46-9B4F-5655A1097276</t>
         </is>
       </c>
       <c r="N40" t="n">
-        <v>38500</v>
+        <v>44000</v>
       </c>
       <c r="O40" t="n">
-        <v>6160</v>
+        <v>7040</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="Q40" t="n">
-        <v>44660</v>
+        <v>49280</v>
       </c>
     </row>
     <row r="41">
@@ -3253,40 +3248,40 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>D143134</t>
+          <t>FM013591</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>DEMORAS</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>8213514F-CC1A-45DF-BCAF-51C56A75D75B</t>
+          <t>BA8E4D43-500F-614F-815A-935A4AA73678</t>
         </is>
       </c>
       <c r="N41" t="n">
-        <v>10500</v>
+        <v>44000</v>
       </c>
       <c r="O41" t="n">
-        <v>1680</v>
+        <v>7040</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="Q41" t="n">
-        <v>10500</v>
+        <v>49280</v>
       </c>
     </row>
     <row r="42">
@@ -3322,40 +3317,40 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>D143134</t>
+          <t>FM013648</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ESTADIAS</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>6E45A124-CBB9-401B-9501-48BEA9E4E82F</t>
+          <t>8CCE2D32-B553-354A-BC06-82B7A4BB3BCF</t>
         </is>
       </c>
       <c r="N42" t="n">
-        <v>2418</v>
+        <v>38500</v>
       </c>
       <c r="O42" t="n">
-        <v>386.88</v>
+        <v>6160</v>
       </c>
       <c r="P42" t="n">
         <v>0</v>
       </c>
       <c r="Q42" t="n">
-        <v>2418</v>
+        <v>44660</v>
       </c>
     </row>
     <row r="43">
@@ -3391,40 +3386,40 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>D143134</t>
+          <t>FM013649</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>ESTADIAS</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>d2dcda60-647e-4c01-b87a-7fcf74d67605</t>
+          <t>103BB1B9-B764-D245-BAA7-3A9B0C7B44DC</t>
         </is>
       </c>
       <c r="N43" t="n">
-        <v>40335.44</v>
+        <v>38500</v>
       </c>
       <c r="O43" t="n">
-        <v>6453.67</v>
+        <v>6160</v>
       </c>
       <c r="P43" t="n">
         <v>0</v>
       </c>
       <c r="Q43" t="n">
-        <v>40335.44</v>
+        <v>44660</v>
       </c>
     </row>
     <row r="44">
@@ -3460,7 +3455,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3475,25 +3470,25 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>DEMORAS</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>7e1d0a34-db4b-4bbf-9ed7-295b32d0858d</t>
+          <t>8213514F-CC1A-45DF-BCAF-51C56A75D75B</t>
         </is>
       </c>
       <c r="N44" t="n">
-        <v>40335.44</v>
+        <v>10500</v>
       </c>
       <c r="O44" t="n">
-        <v>6453.67</v>
+        <v>1680</v>
       </c>
       <c r="P44" t="n">
         <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>40335.44</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="45">
@@ -3529,7 +3524,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -3547,17 +3542,22 @@
           <t>DESCONSOLIDACION</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>6E45A124-CBB9-401B-9501-48BEA9E4E82F</t>
+        </is>
+      </c>
       <c r="N45" t="n">
-        <v>1395</v>
+        <v>2418</v>
       </c>
       <c r="O45" t="n">
-        <v>223.2</v>
+        <v>386.88</v>
       </c>
       <c r="P45" t="n">
         <v>0</v>
       </c>
       <c r="Q45" t="n">
-        <v>1395</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="46">
@@ -3613,20 +3613,20 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>5EB26B13-B1B0-560D-865B-EADC452AA2B7</t>
+          <t>d2dcda60-647e-4c01-b87a-7fcf74d67605</t>
         </is>
       </c>
       <c r="N46" t="n">
-        <v>5300</v>
+        <v>40335.44</v>
       </c>
       <c r="O46" t="n">
-        <v>848</v>
+        <v>6453.67</v>
       </c>
       <c r="P46" t="n">
         <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>5300</v>
+        <v>40335.44</v>
       </c>
     </row>
     <row r="47">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>26/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3682,20 +3682,20 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>D5DD9776-5246-5C11-88DF-5001C3E4C068</t>
+          <t>7e1d0a34-db4b-4bbf-9ed7-295b32d0858d</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>1200</v>
+        <v>40335.44</v>
       </c>
       <c r="O47" t="n">
-        <v>192</v>
+        <v>6453.67</v>
       </c>
       <c r="P47" t="n">
         <v>0</v>
       </c>
       <c r="Q47" t="n">
-        <v>1200</v>
+        <v>40335.44</v>
       </c>
     </row>
     <row r="48">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3746,25 +3746,20 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>E0A74DA2-3EC7-5C4D-A02D-73C8C95E7453</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="N48" t="n">
-        <v>5300</v>
+        <v>1395</v>
       </c>
       <c r="O48" t="n">
-        <v>848</v>
+        <v>223.2</v>
       </c>
       <c r="P48" t="n">
         <v>0</v>
       </c>
       <c r="Q48" t="n">
-        <v>5300</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="49">
@@ -3800,7 +3795,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3815,20 +3810,25 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>5EB26B13-B1B0-560D-865B-EADC452AA2B7</t>
         </is>
       </c>
       <c r="N49" t="n">
-        <v>446.4</v>
+        <v>5300</v>
       </c>
       <c r="O49" t="n">
-        <v>0</v>
+        <v>848</v>
       </c>
       <c r="P49" t="n">
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>446.4</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="50">
@@ -3884,20 +3884,20 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>3F123E87-3748-51E0-9888-1EA1790F1A13</t>
+          <t>D5DD9776-5246-5C11-88DF-5001C3E4C068</t>
         </is>
       </c>
       <c r="N50" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="O50" t="n">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="P50" t="n">
         <v>0</v>
       </c>
       <c r="Q50" t="n">
-        <v>600</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="51">
@@ -3933,40 +3933,40 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>A45782</t>
+          <t>D143134</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>HONORARIOS DE AGENCIA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>c8941213-a088-434b-bb39-744c6cbe2668</t>
+          <t>E0A74DA2-3EC7-5C4D-A02D-73C8C95E7453</t>
         </is>
       </c>
       <c r="N51" t="n">
-        <v>283883.88</v>
+        <v>5300</v>
       </c>
       <c r="O51" t="n">
-        <v>45421.42</v>
+        <v>848</v>
       </c>
       <c r="P51" t="n">
         <v>0</v>
       </c>
       <c r="Q51" t="n">
-        <v>329305.3</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="52">
@@ -3987,12 +3987,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>MNSI262347</t>
+          <t>MNSI261767</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>6003509</t>
+          <t>6002723</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4002,40 +4002,35 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>A57791</t>
+          <t>D143134</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>DC76827C-991A-4D5B-A922-4D221EAF5235</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="N52" t="n">
-        <v>3250</v>
+        <v>446.4</v>
       </c>
       <c r="O52" t="n">
-        <v>520</v>
+        <v>0</v>
       </c>
       <c r="P52" t="n">
         <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>3770</v>
+        <v>446.4</v>
       </c>
     </row>
     <row r="53">
@@ -4056,12 +4051,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MNSI262347</t>
+          <t>MNSI261767</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>6003509</t>
+          <t>6002723</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4071,35 +4066,40 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>26/03/2026</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>3134454050</t>
+          <t>D143134</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>DHL EXPRESS MEXICO S.A. DE C.V</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>MENSAJERIA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>3F123E87-3748-51E0-9888-1EA1790F1A13</t>
         </is>
       </c>
       <c r="N53" t="n">
-        <v>349.04</v>
+        <v>600</v>
       </c>
       <c r="O53" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="P53" t="n">
         <v>0</v>
       </c>
       <c r="Q53" t="n">
-        <v>349.04</v>
+        <v>600</v>
       </c>
     </row>
     <row r="54">
@@ -4120,12 +4120,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MNSI262347</t>
+          <t>MNSI261767</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>6003509</t>
+          <t>6002723</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4135,40 +4135,40 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>FM013632</t>
+          <t>A45782</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>7758E8C3-A8AE-F54E-95FD-72ED5DE7AC31</t>
+          <t>c8941213-a088-434b-bb39-744c6cbe2668</t>
         </is>
       </c>
       <c r="N54" t="n">
-        <v>53000</v>
+        <v>283883.88</v>
       </c>
       <c r="O54" t="n">
-        <v>8480</v>
+        <v>45421.42</v>
       </c>
       <c r="P54" t="n">
-        <v>2120</v>
+        <v>0</v>
       </c>
       <c r="Q54" t="n">
-        <v>59360</v>
+        <v>329305.3</v>
       </c>
     </row>
     <row r="55">
@@ -4204,40 +4204,40 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>D143783</t>
+          <t>A57791</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>5A05D33A-6240-4739-AA50-F6B4547C9A26</t>
+          <t>DC76827C-991A-4D5B-A922-4D221EAF5235</t>
         </is>
       </c>
       <c r="N55" t="n">
-        <v>2865.51</v>
+        <v>3250</v>
       </c>
       <c r="O55" t="n">
-        <v>458.48</v>
+        <v>520</v>
       </c>
       <c r="P55" t="n">
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>2865.51</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="56">
@@ -4273,40 +4273,35 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>D143783</t>
+          <t>3134454050</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>DHL EXPRESS MEXICO S.A. DE C.V</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>9E7FE2B1-3A5D-40F6-8CB4-B7A10C961BA6</t>
+          <t>MENSAJERIA</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>8101.59</v>
+        <v>349.04</v>
       </c>
       <c r="O56" t="n">
-        <v>1296.25</v>
+        <v>0</v>
       </c>
       <c r="P56" t="n">
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>8101.59</v>
+        <v>349.04</v>
       </c>
     </row>
     <row r="57">
@@ -4342,40 +4337,40 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>D143783</t>
+          <t>FM013632</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES VIKINGO SA DE CV</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>4F0E2F90-26C0-4BC8-9521-EFD02B5BEEA6</t>
+          <t>7758E8C3-A8AE-F54E-95FD-72ED5DE7AC31</t>
         </is>
       </c>
       <c r="N57" t="n">
-        <v>3615</v>
+        <v>53000</v>
       </c>
       <c r="O57" t="n">
-        <v>578.4</v>
+        <v>8480</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>2120</v>
       </c>
       <c r="Q57" t="n">
-        <v>3615</v>
+        <v>59360</v>
       </c>
     </row>
     <row r="58">
@@ -4411,7 +4406,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4431,20 +4426,20 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>929D3848-CA92-409A-91BF-7358EBA1339E</t>
+          <t>5A05D33A-6240-4739-AA50-F6B4547C9A26</t>
         </is>
       </c>
       <c r="N58" t="n">
-        <v>8487.389999999999</v>
+        <v>2865.51</v>
       </c>
       <c r="O58" t="n">
-        <v>1357.98</v>
+        <v>458.48</v>
       </c>
       <c r="P58" t="n">
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>8487.389999999999</v>
+        <v>2865.51</v>
       </c>
     </row>
     <row r="59">
@@ -4480,7 +4475,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -4500,20 +4495,20 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>0031D53A-AEA9-4B7E-B98B-0A1242C40A85</t>
+          <t>9E7FE2B1-3A5D-40F6-8CB4-B7A10C961BA6</t>
         </is>
       </c>
       <c r="N59" t="n">
-        <v>5658.26</v>
+        <v>8101.59</v>
       </c>
       <c r="O59" t="n">
-        <v>905.3200000000001</v>
+        <v>1296.25</v>
       </c>
       <c r="P59" t="n">
         <v>0</v>
       </c>
       <c r="Q59" t="n">
-        <v>5658.26</v>
+        <v>8101.59</v>
       </c>
     </row>
     <row r="60">
@@ -4549,7 +4544,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -4569,20 +4564,20 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>8C337418-DC79-49AF-9D01-63003E4657DF</t>
+          <t>4F0E2F90-26C0-4BC8-9521-EFD02B5BEEA6</t>
         </is>
       </c>
       <c r="N60" t="n">
-        <v>17907.08</v>
+        <v>3615</v>
       </c>
       <c r="O60" t="n">
-        <v>2865.13</v>
+        <v>578.4</v>
       </c>
       <c r="P60" t="n">
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>17907.08</v>
+        <v>3615</v>
       </c>
     </row>
     <row r="61">
@@ -4618,7 +4613,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -4638,20 +4633,20 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>532C622D-98E1-5040-B626-59030A9598FD</t>
+          <t>929D3848-CA92-409A-91BF-7358EBA1339E</t>
         </is>
       </c>
       <c r="N61" t="n">
-        <v>5800</v>
+        <v>8487.389999999999</v>
       </c>
       <c r="O61" t="n">
-        <v>928</v>
+        <v>1357.98</v>
       </c>
       <c r="P61" t="n">
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>5800</v>
+        <v>8487.389999999999</v>
       </c>
     </row>
     <row r="62">
@@ -4687,7 +4682,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -4702,25 +4697,25 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>556B3BAC-ED72-43AC-9B97-9B9D2C51A3AA</t>
+          <t>0031D53A-AEA9-4B7E-B98B-0A1242C40A85</t>
         </is>
       </c>
       <c r="N62" t="n">
-        <v>5329.5</v>
+        <v>5658.26</v>
       </c>
       <c r="O62" t="n">
-        <v>0</v>
+        <v>905.3200000000001</v>
       </c>
       <c r="P62" t="n">
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>5329.5</v>
+        <v>5658.26</v>
       </c>
     </row>
     <row r="63">
@@ -4756,40 +4751,40 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>A46196</t>
+          <t>D143783</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>HONORARIOS DE AGENCIA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>caacf212-989d-43bb-8ef0-430436add959</t>
+          <t>8C337418-DC79-49AF-9D01-63003E4657DF</t>
         </is>
       </c>
       <c r="N63" t="n">
-        <v>114033.87</v>
+        <v>17907.08</v>
       </c>
       <c r="O63" t="n">
-        <v>18245.41</v>
+        <v>2865.13</v>
       </c>
       <c r="P63" t="n">
         <v>0</v>
       </c>
       <c r="Q63" t="n">
-        <v>132279.28</v>
+        <v>17907.08</v>
       </c>
     </row>
     <row r="64">
@@ -4810,12 +4805,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MNSI263354</t>
+          <t>MNSI262347</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>6004737</t>
+          <t>6003509</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4825,40 +4820,40 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>A58816</t>
+          <t>D143783</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>3F2F411A-6DDE-42E3-97FD-C9F3E3E7CBFD</t>
+          <t>532C622D-98E1-5040-B626-59030A9598FD</t>
         </is>
       </c>
       <c r="N64" t="n">
-        <v>6500</v>
+        <v>5800</v>
       </c>
       <c r="O64" t="n">
-        <v>1040</v>
+        <v>928</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>7540</v>
+        <v>5800</v>
       </c>
     </row>
     <row r="65">
@@ -4879,12 +4874,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>MNSI263354</t>
+          <t>MNSI262347</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>6004737</t>
+          <t>6003509</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -4894,40 +4889,40 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>FM002954</t>
+          <t>D143783</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES KARVE</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>3C029339-F000-7B43-8C0F-263155603B0B</t>
+          <t>556B3BAC-ED72-43AC-9B97-9B9D2C51A3AA</t>
         </is>
       </c>
       <c r="N65" t="n">
-        <v>44000</v>
+        <v>5329.5</v>
       </c>
       <c r="O65" t="n">
-        <v>7040</v>
+        <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>1760</v>
+        <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>49280</v>
+        <v>5329.5</v>
       </c>
     </row>
     <row r="66">
@@ -4948,12 +4943,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MNSI263354</t>
+          <t>MNSI262347</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>6004737</t>
+          <t>6003509</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4963,40 +4958,40 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>FM002958</t>
+          <t>A46196</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES KARVE</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>ESTADIAS</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>3B803A06-4795-5243-8C0D-CB165F58BC39</t>
+          <t>caacf212-989d-43bb-8ef0-430436add959</t>
         </is>
       </c>
       <c r="N66" t="n">
-        <v>5500</v>
+        <v>114033.87</v>
       </c>
       <c r="O66" t="n">
-        <v>880</v>
+        <v>18245.41</v>
       </c>
       <c r="P66" t="n">
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>6380</v>
+        <v>132279.28</v>
       </c>
     </row>
     <row r="67">
@@ -5032,40 +5027,40 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>FM002959</t>
+          <t>A58816</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES KARVE</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>ESTADIAS</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>0D2D7C40-86C6-5B43-8A0F-B9F868511EDB</t>
+          <t>3F2F411A-6DDE-42E3-97FD-C9F3E3E7CBFD</t>
         </is>
       </c>
       <c r="N67" t="n">
-        <v>5500</v>
+        <v>6500</v>
       </c>
       <c r="O67" t="n">
-        <v>880</v>
+        <v>1040</v>
       </c>
       <c r="P67" t="n">
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>6380</v>
+        <v>7540</v>
       </c>
     </row>
     <row r="68">
@@ -5106,7 +5101,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>FM002955</t>
+          <t>FM002954</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5121,7 +5116,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>7CF484C6-E361-EA40-A102-555D8C163028</t>
+          <t>3C029339-F000-7B43-8C0F-263155603B0B</t>
         </is>
       </c>
       <c r="N68" t="n">
@@ -5170,40 +5165,40 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>D145100</t>
+          <t>FM002958</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES KARVE</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>ESTADIAS</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>64A224C0-BE42-5635-820B-FF33195AE72E</t>
+          <t>3B803A06-4795-5243-8C0D-CB165F58BC39</t>
         </is>
       </c>
       <c r="N69" t="n">
-        <v>5300</v>
+        <v>5500</v>
       </c>
       <c r="O69" t="n">
-        <v>848</v>
+        <v>880</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>5300</v>
+        <v>6380</v>
       </c>
     </row>
     <row r="70">
@@ -5239,40 +5234,40 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>D145100</t>
+          <t>FM002959</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES KARVE</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>ESTADIAS</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>6A39880E-7FCD-5221-B8D9-34F4BF9EE9A1</t>
+          <t>0D2D7C40-86C6-5B43-8A0F-B9F868511EDB</t>
         </is>
       </c>
       <c r="N70" t="n">
-        <v>5300</v>
+        <v>5500</v>
       </c>
       <c r="O70" t="n">
-        <v>848</v>
+        <v>880</v>
       </c>
       <c r="P70" t="n">
         <v>0</v>
       </c>
       <c r="Q70" t="n">
-        <v>5300</v>
+        <v>6380</v>
       </c>
     </row>
     <row r="71">
@@ -5308,40 +5303,40 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>D145100</t>
+          <t>FM002955</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES KARVE</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>E24E29EF-76D8-4EE5-9AEB-DC3F636FAB11</t>
+          <t>7CF484C6-E361-EA40-A102-555D8C163028</t>
         </is>
       </c>
       <c r="N71" t="n">
-        <v>16144</v>
+        <v>44000</v>
       </c>
       <c r="O71" t="n">
-        <v>2583.04</v>
+        <v>7040</v>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="Q71" t="n">
-        <v>16144</v>
+        <v>49280</v>
       </c>
     </row>
     <row r="72">
@@ -5377,7 +5372,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -5397,20 +5392,20 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>596FB89B-A6A6-4104-A84B-52B81A841A18</t>
+          <t>64A224C0-BE42-5635-820B-FF33195AE72E</t>
         </is>
       </c>
       <c r="N72" t="n">
-        <v>19803.91</v>
+        <v>5300</v>
       </c>
       <c r="O72" t="n">
-        <v>3168.63</v>
+        <v>848</v>
       </c>
       <c r="P72" t="n">
         <v>0</v>
       </c>
       <c r="Q72" t="n">
-        <v>19803.91</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="73">
@@ -5446,7 +5441,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -5466,20 +5461,20 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>3A52C365-D527-469E-972E-5DE727DB19CE</t>
+          <t>6A39880E-7FCD-5221-B8D9-34F4BF9EE9A1</t>
         </is>
       </c>
       <c r="N73" t="n">
-        <v>23546.37</v>
+        <v>5300</v>
       </c>
       <c r="O73" t="n">
-        <v>3767.42</v>
+        <v>848</v>
       </c>
       <c r="P73" t="n">
         <v>0</v>
       </c>
       <c r="Q73" t="n">
-        <v>23546.37</v>
+        <v>5300</v>
       </c>
     </row>
     <row r="74">
@@ -5515,7 +5510,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -5535,20 +5530,20 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>CC64CDE8-382A-4F1B-B356-C740E880F26B</t>
+          <t>E24E29EF-76D8-4EE5-9AEB-DC3F636FAB11</t>
         </is>
       </c>
       <c r="N74" t="n">
-        <v>16203.18</v>
+        <v>16144</v>
       </c>
       <c r="O74" t="n">
-        <v>2592.51</v>
+        <v>2583.04</v>
       </c>
       <c r="P74" t="n">
         <v>0</v>
       </c>
       <c r="Q74" t="n">
-        <v>16203.18</v>
+        <v>16144</v>
       </c>
     </row>
     <row r="75">
@@ -5584,7 +5579,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -5604,20 +5599,20 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>04F0DFEA-465F-432C-B65C-A8FDEAA5212A</t>
+          <t>596FB89B-A6A6-4104-A84B-52B81A841A18</t>
         </is>
       </c>
       <c r="N75" t="n">
-        <v>8873.16</v>
+        <v>19803.91</v>
       </c>
       <c r="O75" t="n">
-        <v>1419.71</v>
+        <v>3168.63</v>
       </c>
       <c r="P75" t="n">
         <v>0</v>
       </c>
       <c r="Q75" t="n">
-        <v>8873.16</v>
+        <v>19803.91</v>
       </c>
     </row>
     <row r="76">
@@ -5653,7 +5648,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -5673,20 +5668,20 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>7429B256-3C80-4B24-8377-87D1DB11D476</t>
+          <t>3A52C365-D527-469E-972E-5DE727DB19CE</t>
         </is>
       </c>
       <c r="N76" t="n">
-        <v>8487.389999999999</v>
+        <v>23546.37</v>
       </c>
       <c r="O76" t="n">
-        <v>1357.98</v>
+        <v>3767.42</v>
       </c>
       <c r="P76" t="n">
         <v>0</v>
       </c>
       <c r="Q76" t="n">
-        <v>8487.389999999999</v>
+        <v>23546.37</v>
       </c>
     </row>
     <row r="77">
@@ -5722,7 +5717,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -5742,20 +5737,20 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>5AF62066-157C-45AA-93DB-9F2361DB8FC6</t>
+          <t>CC64CDE8-382A-4F1B-B356-C740E880F26B</t>
         </is>
       </c>
       <c r="N77" t="n">
-        <v>2865.51</v>
+        <v>16203.18</v>
       </c>
       <c r="O77" t="n">
-        <v>458.48</v>
+        <v>2592.51</v>
       </c>
       <c r="P77" t="n">
         <v>0</v>
       </c>
       <c r="Q77" t="n">
-        <v>2865.51</v>
+        <v>16203.18</v>
       </c>
     </row>
     <row r="78">
@@ -5791,7 +5786,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -5811,20 +5806,20 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>1A2FEA54-D3D2-48B2-8F94-03A5D7BA6C19</t>
+          <t>04F0DFEA-465F-432C-B65C-A8FDEAA5212A</t>
         </is>
       </c>
       <c r="N78" t="n">
-        <v>2865.51</v>
+        <v>8873.16</v>
       </c>
       <c r="O78" t="n">
-        <v>458.48</v>
+        <v>1419.71</v>
       </c>
       <c r="P78" t="n">
         <v>0</v>
       </c>
       <c r="Q78" t="n">
-        <v>2865.51</v>
+        <v>8873.16</v>
       </c>
     </row>
     <row r="79">
@@ -5860,7 +5855,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -5875,20 +5870,25 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>7429B256-3C80-4B24-8377-87D1DB11D476</t>
         </is>
       </c>
       <c r="N79" t="n">
-        <v>547.5</v>
+        <v>8487.389999999999</v>
       </c>
       <c r="O79" t="n">
-        <v>87.59999999999999</v>
+        <v>1357.98</v>
       </c>
       <c r="P79" t="n">
         <v>0</v>
       </c>
       <c r="Q79" t="n">
-        <v>635.1</v>
+        <v>8487.389999999999</v>
       </c>
     </row>
     <row r="80">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -5939,20 +5939,25 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>5AF62066-157C-45AA-93DB-9F2361DB8FC6</t>
         </is>
       </c>
       <c r="N80" t="n">
-        <v>8212.5</v>
+        <v>2865.51</v>
       </c>
       <c r="O80" t="n">
-        <v>0</v>
+        <v>458.48</v>
       </c>
       <c r="P80" t="n">
         <v>0</v>
       </c>
       <c r="Q80" t="n">
-        <v>8212.5</v>
+        <v>2865.51</v>
       </c>
     </row>
     <row r="81">
@@ -5988,40 +5993,40 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>29/06/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>A47861</t>
+          <t>D145100</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>HONORARIOS DE AGENCIA</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>54eefdf9-a847-4a9e-92b4-3bd7f6724d2a</t>
+          <t>1A2FEA54-D3D2-48B2-8F94-03A5D7BA6C19</t>
         </is>
       </c>
       <c r="N81" t="n">
-        <v>224889.03</v>
+        <v>2865.51</v>
       </c>
       <c r="O81" t="n">
-        <v>35982.25</v>
+        <v>458.48</v>
       </c>
       <c r="P81" t="n">
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>260871.28</v>
+        <v>2865.51</v>
       </c>
     </row>
     <row r="82">
@@ -6042,12 +6047,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>MNSI263710</t>
+          <t>MNSI263354</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>6005334</t>
+          <t>6004737</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6057,40 +6062,35 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>24/06/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>A59027</t>
+          <t>D145100</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>MANIOBRAS DE DESCARGA</t>
-        </is>
-      </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>5DE651A2-8064-4A9F-91C9-83F9496B666A</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="N82" t="n">
-        <v>6500</v>
+        <v>547.5</v>
       </c>
       <c r="O82" t="n">
-        <v>1040</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="P82" t="n">
         <v>0</v>
       </c>
       <c r="Q82" t="n">
-        <v>7540</v>
+        <v>635.1</v>
       </c>
     </row>
     <row r="83">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>MNSI263710</t>
+          <t>MNSI263354</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>6005334</t>
+          <t>6004737</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -6126,40 +6126,35 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>08/06/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>FM003030</t>
+          <t>D145100</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES KARVE</t>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
-        </is>
-      </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>A7ED86D8-5BBE-1D49-87AF-B2A7EA5B2BD4</t>
+          <t>DESCONSOLIDACION</t>
         </is>
       </c>
       <c r="N83" t="n">
-        <v>44000</v>
+        <v>8212.5</v>
       </c>
       <c r="O83" t="n">
-        <v>7040</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>1760</v>
+        <v>0</v>
       </c>
       <c r="Q83" t="n">
-        <v>49280</v>
+        <v>8212.5</v>
       </c>
     </row>
     <row r="84">
@@ -6180,12 +6175,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>MNSI263710</t>
+          <t>MNSI263354</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>6005334</t>
+          <t>6004737</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -6195,40 +6190,40 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>08/06/2026</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>FM003031</t>
+          <t>A47861</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>AUTOTRANSPORTES KARVE</t>
+          <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>FLETE TERRESTRE</t>
+          <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>7B0BC44F-F8A9-B24E-B063-4310EE36651F</t>
+          <t>54eefdf9-a847-4a9e-92b4-3bd7f6724d2a</t>
         </is>
       </c>
       <c r="N84" t="n">
-        <v>44000</v>
+        <v>224889.03</v>
       </c>
       <c r="O84" t="n">
-        <v>7040</v>
+        <v>35982.25</v>
       </c>
       <c r="P84" t="n">
-        <v>1760</v>
+        <v>0</v>
       </c>
       <c r="Q84" t="n">
-        <v>49280</v>
+        <v>260871.28</v>
       </c>
     </row>
     <row r="85">
@@ -6264,40 +6259,40 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>D145699</t>
+          <t>A59027</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>SUPER EXPRESS DE CARGA FEDERAL S.A. DE C.V.</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>MANIOBRAS DE DESCARGA</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>b833b5df-76ab-47d1-8860-a34b12a4bce5</t>
+          <t>5DE651A2-8064-4A9F-91C9-83F9496B666A</t>
         </is>
       </c>
       <c r="N85" t="n">
-        <v>43096.28</v>
+        <v>6500</v>
       </c>
       <c r="O85" t="n">
-        <v>6895.4</v>
+        <v>1040</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
       </c>
       <c r="Q85" t="n">
-        <v>43096.28</v>
+        <v>7540</v>
       </c>
     </row>
     <row r="86">
@@ -6333,40 +6328,40 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>D145699</t>
+          <t>FM003030</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES KARVE</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>03f42c61-253a-4e0e-a95d-221d71090397</t>
+          <t>A7ED86D8-5BBE-1D49-87AF-B2A7EA5B2BD4</t>
         </is>
       </c>
       <c r="N86" t="n">
-        <v>45857.12</v>
+        <v>44000</v>
       </c>
       <c r="O86" t="n">
-        <v>7337.14</v>
+        <v>7040</v>
       </c>
       <c r="P86" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="Q86" t="n">
-        <v>45857.12</v>
+        <v>49280</v>
       </c>
     </row>
     <row r="87">
@@ -6402,40 +6397,40 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>D145699</t>
+          <t>FM003031</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+          <t>AUTOTRANSPORTES KARVE</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+          <t>FLETE TERRESTRE</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>290DA40C-06A8-5CD9-A59C-69BB508F250B</t>
+          <t>7B0BC44F-F8A9-B24E-B063-4310EE36651F</t>
         </is>
       </c>
       <c r="N87" t="n">
-        <v>5850</v>
+        <v>44000</v>
       </c>
       <c r="O87" t="n">
-        <v>936</v>
+        <v>7040</v>
       </c>
       <c r="P87" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="Q87" t="n">
-        <v>5850</v>
+        <v>49280</v>
       </c>
     </row>
     <row r="88">
@@ -6471,7 +6466,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -6491,20 +6486,20 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>3FB5D676-55FD-5277-85AB-8227156C3DED</t>
+          <t>b833b5df-76ab-47d1-8860-a34b12a4bce5</t>
         </is>
       </c>
       <c r="N88" t="n">
-        <v>5850</v>
+        <v>43096.28</v>
       </c>
       <c r="O88" t="n">
-        <v>936</v>
+        <v>6895.4</v>
       </c>
       <c r="P88" t="n">
         <v>0</v>
       </c>
       <c r="Q88" t="n">
-        <v>5850</v>
+        <v>43096.28</v>
       </c>
     </row>
     <row r="89">
@@ -6540,7 +6535,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -6555,25 +6550,25 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>DESCONSOLIDACION</t>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>B4EE3798-806C-4291-8706-02407EACD745</t>
+          <t>03f42c61-253a-4e0e-a95d-221d71090397</t>
         </is>
       </c>
       <c r="N89" t="n">
-        <v>6605.6</v>
+        <v>45857.12</v>
       </c>
       <c r="O89" t="n">
-        <v>1056.9</v>
+        <v>7337.14</v>
       </c>
       <c r="P89" t="n">
         <v>0</v>
       </c>
       <c r="Q89" t="n">
-        <v>7662.5</v>
+        <v>45857.12</v>
       </c>
     </row>
     <row r="90">
@@ -6609,39 +6604,246 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>D145699</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>290DA40C-06A8-5CD9-A59C-69BB508F250B</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>5850</v>
+      </c>
+      <c r="O90" t="n">
+        <v>936</v>
+      </c>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>5850</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Importación</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MNSI263710</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>6005334</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>D145699</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>ALMACENAJE, MANEJO Y CUSTODIA</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>3FB5D676-55FD-5277-85AB-8227156C3DED</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>5850</v>
+      </c>
+      <c r="O91" t="n">
+        <v>936</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>5850</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Importación</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MNSI263710</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>6005334</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>D145699</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>OÑATE WILLY Y COMPAÑÍA, S.C. (MANZANILLO)</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>DESCONSOLIDACION</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>B4EE3798-806C-4291-8706-02407EACD745</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>6605.6</v>
+      </c>
+      <c r="O92" t="n">
+        <v>1056.9</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>7662.5</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Importación</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SANOFI PASTEUR, S.A DE C.V.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MNSI263710</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>6005334</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
           <t>29/06/2026</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="J93" t="inlineStr">
         <is>
           <t>A47941</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
+      <c r="K93" t="inlineStr">
         <is>
           <t>ABSOLUTE BROKERAGE CUSTOMS, S.C.</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr">
+      <c r="L93" t="inlineStr">
         <is>
           <t>HONORARIOS DE AGENCIA</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr">
+      <c r="M93" t="inlineStr">
         <is>
           <t>91503410-5a3b-4ad2-b497-bd7d01418de3</t>
         </is>
       </c>
-      <c r="N90" t="n">
+      <c r="N93" t="n">
         <v>205153.4</v>
       </c>
-      <c r="O90" t="n">
+      <c r="O93" t="n">
         <v>32824.54</v>
       </c>
-      <c r="P90" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q90" t="n">
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="n">
         <v>237977.94</v>
       </c>
     </row>

</xml_diff>